<commit_message>
chore: publish hospitalnotification IG 3.0.2
</commit_message>
<xml_diff>
--- a/ig/hospitalnotification/StructureDefinition-medcom-hospitalNotification-message.xlsx
+++ b/ig/hospitalnotification/StructureDefinition-medcom-hospitalNotification-message.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1788" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1788" uniqueCount="268">
   <si>
     <t>Property</t>
   </si>
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>3.0.1</t>
+    <t>3.0.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-03-02T09:56:15+01:00</t>
+    <t>2026-02-10T12:55:02+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -69,7 +69,7 @@
     <t>Contact</t>
   </si>
   <si>
-    <t>No display for ContactDetail</t>
+    <t>MedCom (http://www.medcom.dk)</t>
   </si>
   <si>
     <t>Jurisdiction</t>
@@ -263,6 +263,10 @@
   </si>
   <si>
     <t>A container for a collection of resources.</t>
+  </si>
+  <si>
+    <t>bdl-1:total only when a search or history {total.empty() or (type = 'searchset') or (type = 'history')}
+bdl-2:entry.search only when a search {entry.search.empty() or (type = 'searchset')}bdl-3:entry.request mandatory for batch/transaction/history, otherwise prohibited {entry.all(request.exists() = (%resource.type = 'batch' or %resource.type = 'transaction' or %resource.type = 'history'))}bdl-4:entry.response mandatory for batch-response/transaction-response/history, otherwise prohibited {entry.all(response.exists() = (%resource.type = 'batch-response' or %resource.type = 'transaction-response' or %resource.type = 'history'))}bdl-7:FullUrl must be unique in a bundle, or else entries with the same fullUrl must have different meta.versionId (except in history bundles) {(type = 'history') or entry.where(fullUrl.exists()).select(fullUrl&amp;resource.meta.versionId).isDistinct()}bdl-9:A document must have an identifier with a system and a value {type = 'document' implies (identifier.system.exists() and identifier.value.exists())}bdl-10:A document must have a date {type = 'document' implies (timestamp.hasValue())}bdl-11:A document must have a Composition as the first resource {type = 'document' implies entry.first().resource.is(Composition)}bdl-12:A message must have a MessageHeader as the first resource {type = 'message' implies entry.first().resource.is(MessageHeader)}medcom-messaging-1:The MessageHeader resource shall conform to medcom-messaging-messageHeader profile {entry.ofType(MessageHeader).all(resource.conformsTo('http://medcomfhir.dk/fhir/messaging/StructureDefinition/medcom-messaging-messageHeader'))}medcom-messaging-2:There shall be at least one Provenance resource in a MedCom message {entry.resource.ofType(Provenance).exists()}medcom-messaging-3:All Provenance resources shall conform to medcom-core-provenance profile {entry.ofType(Provenance).all(resource.conformsTo('http://medcomfhir.dk/fhir/messaging/StructureDefinition/medcom-messaging-provenance'))}medcom-hospitalNotification-1:The message header shall conform to medcom-hospitalNotification-messageHeader profile {entry.ofType(MessageHeader).all(resource.conformsTo('http://medcomfhir.dk/fhir/hospitalnotification/StructureDefinition/medcom-hospitalNotification-messageHeader'))}medcom-hospitalNotification-2:Entry shall contain exactly one patient resource {entry.where(resource.is(Patient)).count() = 1}medcom-hospitalNotification-3:All provenance resources shall contain activities from medcom-hospitalNotification-messageActivities valueset {entry.ofType(Provenance).all(resource.activity.memberOf('http://medcomfhir.dk/fhir/dk-medcom-terminology/ValueSet/medcom-hospitalNotification-messageActivities'))}medcom-hospitalNotification-4:The system of Patient.identifier shall be 'urn:oid:1.2.208.176.1.2', which represents an official Danish CPR-number {entry.resource.ofType(Patient).identifier.system = 'urn:oid:1.2.208.176.1.2'}medcom-hospitalNotification-5:The receiver of a HospitalNotification shall always be a primary receiver. {Bundle.entry.resource.ofType(MessageHeader).destination.extension.value.code = 'primary'}</t>
   </si>
   <si>
     <t>N/A</t>
@@ -976,10 +980,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyBorder="true" applyFill="true" applyFont="true">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyBorder="true" applyFill="true" applyAlignment="true" applyFont="true">
       <alignment vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="true" applyAlignment="true">
       <alignment vertical="top" wrapText="true"/>
     </xf>
   </cellXfs>
@@ -1172,17 +1176,17 @@
   <dimension ref="A1:AN49"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="38.1796875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="38.1796875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.1328125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="4" max="4" width="20.859375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="5" max="5" width="5.90234375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="4.69921875" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="5.07421875" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="14.625" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="11.98828125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="33.44140625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="33.44140625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="4" max="4" width="18.19140625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="4.65625" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="17.203125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="15.140625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -1191,26 +1195,26 @@
     <col min="17" max="17" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="18" max="18" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="19" max="19" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" width="8.84375" customWidth="true" bestFit="true"/>
-    <col min="21" max="21" width="15.71484375" customWidth="true" bestFit="true"/>
-    <col min="22" max="22" width="16.08984375" customWidth="true" bestFit="true"/>
-    <col min="23" max="23" width="17.078125" customWidth="true" bestFit="true"/>
-    <col min="24" max="24" width="16.3125" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="163.2734375" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="49.55078125" customWidth="true" bestFit="true"/>
-    <col min="27" max="27" width="5.69140625" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="19.73046875" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" width="17.8203125" customWidth="true" bestFit="true"/>
-    <col min="30" max="30" width="14.98828125" customWidth="true" bestFit="true"/>
-    <col min="31" max="31" width="12.3046875" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="34.5859375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="33" max="33" width="9.5" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="34" max="34" width="9.87890625" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" width="8.53515625" customWidth="true" bestFit="true"/>
+    <col min="21" max="21" width="14.72265625" customWidth="true" bestFit="true"/>
+    <col min="22" max="22" width="15.13671875" customWidth="true" bestFit="true"/>
+    <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
+    <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="144.1953125" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="42.01953125" customWidth="true" bestFit="true"/>
+    <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
+    <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
+    <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="29.98828125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
-    <col min="37" max="37" width="25.01171875" customWidth="true" bestFit="true"/>
-    <col min="38" max="38" width="22.67578125" customWidth="true" bestFit="true"/>
-    <col min="39" max="39" width="41.43359375" customWidth="true" bestFit="true"/>
-    <col min="40" max="40" width="32.84375" customWidth="true" bestFit="true"/>
+    <col min="37" max="37" width="24.1328125" customWidth="true" bestFit="true"/>
+    <col min="38" max="38" width="21.4140625" customWidth="true" bestFit="true"/>
+    <col min="39" max="39" width="36.84375" customWidth="true" bestFit="true"/>
+    <col min="40" max="40" width="31.65234375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1432,27 +1436,27 @@
         <v>76</v>
       </c>
       <c r="AJ2" t="s" s="2">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="AK2" t="s" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AL2" t="s" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AM2" t="s" s="2">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AN2" t="s" s="2">
         <v>76</v>
       </c>
     </row>
-    <row r="3" hidden="true">
+    <row r="3">
       <c r="A3" t="s" s="2">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" t="s" s="2">
@@ -1460,31 +1464,31 @@
       </c>
       <c r="E3" s="2"/>
       <c r="F3" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G3" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H3" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I3" t="s" s="2">
         <v>76</v>
       </c>
       <c r="J3" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K3" t="s" s="2">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L3" t="s" s="2">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="M3" t="s" s="2">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="N3" t="s" s="2">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O3" s="2"/>
       <c r="P3" t="s" s="2">
@@ -1534,13 +1538,13 @@
         <v>76</v>
       </c>
       <c r="AF3" t="s" s="2">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="AG3" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH3" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI3" t="s" s="2">
         <v>76</v>
@@ -1563,10 +1567,10 @@
     </row>
     <row r="4" hidden="true">
       <c r="A4" t="s" s="2">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" t="s" s="2">
@@ -1577,7 +1581,7 @@
         <v>77</v>
       </c>
       <c r="G4" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H4" t="s" s="2">
         <v>76</v>
@@ -1586,16 +1590,16 @@
         <v>76</v>
       </c>
       <c r="J4" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K4" t="s" s="2">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L4" t="s" s="2">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="M4" t="s" s="2">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
@@ -1646,19 +1650,19 @@
         <v>76</v>
       </c>
       <c r="AF4" t="s" s="2">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AG4" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH4" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI4" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ4" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK4" t="s" s="2">
         <v>76</v>
@@ -1675,10 +1679,10 @@
     </row>
     <row r="5" hidden="true">
       <c r="A5" t="s" s="2">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" t="s" s="2">
@@ -1689,28 +1693,28 @@
         <v>77</v>
       </c>
       <c r="G5" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H5" t="s" s="2">
         <v>76</v>
       </c>
       <c r="I5" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J5" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K5" t="s" s="2">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L5" t="s" s="2">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M5" t="s" s="2">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="N5" t="s" s="2">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="O5" s="2"/>
       <c r="P5" t="s" s="2">
@@ -1760,19 +1764,19 @@
         <v>76</v>
       </c>
       <c r="AF5" t="s" s="2">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AG5" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH5" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI5" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ5" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK5" t="s" s="2">
         <v>76</v>
@@ -1789,10 +1793,10 @@
     </row>
     <row r="6" hidden="true">
       <c r="A6" t="s" s="2">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" t="s" s="2">
@@ -1803,7 +1807,7 @@
         <v>77</v>
       </c>
       <c r="G6" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H6" t="s" s="2">
         <v>76</v>
@@ -1815,16 +1819,16 @@
         <v>76</v>
       </c>
       <c r="K6" t="s" s="2">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L6" t="s" s="2">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M6" t="s" s="2">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N6" t="s" s="2">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="O6" s="2"/>
       <c r="P6" t="s" s="2">
@@ -1850,13 +1854,13 @@
         <v>76</v>
       </c>
       <c r="X6" t="s" s="2">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="Y6" t="s" s="2">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="Z6" t="s" s="2">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="AA6" t="s" s="2">
         <v>76</v>
@@ -1874,19 +1878,19 @@
         <v>76</v>
       </c>
       <c r="AF6" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AG6" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH6" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI6" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ6" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK6" t="s" s="2">
         <v>76</v>
@@ -1903,10 +1907,10 @@
     </row>
     <row r="7" hidden="true">
       <c r="A7" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" t="s" s="2">
@@ -1917,7 +1921,7 @@
         <v>77</v>
       </c>
       <c r="G7" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H7" t="s" s="2">
         <v>76</v>
@@ -1926,19 +1930,19 @@
         <v>76</v>
       </c>
       <c r="J7" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K7" t="s" s="2">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="L7" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="M7" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="N7" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="O7" s="2"/>
       <c r="P7" t="s" s="2">
@@ -1988,19 +1992,19 @@
         <v>76</v>
       </c>
       <c r="AF7" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH7" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI7" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ7" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK7" t="s" s="2">
         <v>76</v>
@@ -2009,18 +2013,18 @@
         <v>76</v>
       </c>
       <c r="AM7" t="s" s="2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AN7" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
-    <row r="8" hidden="true">
+    <row r="8">
       <c r="A8" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -2028,31 +2032,31 @@
       </c>
       <c r="E8" s="2"/>
       <c r="F8" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G8" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H8" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I8" t="s" s="2">
         <v>76</v>
       </c>
       <c r="J8" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K8" t="s" s="2">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L8" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M8" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N8" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="O8" s="2"/>
       <c r="P8" t="s" s="2">
@@ -2063,7 +2067,7 @@
         <v>76</v>
       </c>
       <c r="S8" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="T8" t="s" s="2">
         <v>76</v>
@@ -2078,13 +2082,13 @@
         <v>76</v>
       </c>
       <c r="X8" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Y8" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Z8" t="s" s="2">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AA8" t="s" s="2">
         <v>76</v>
@@ -2102,19 +2106,19 @@
         <v>76</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AG8" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AH8" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI8" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ8" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK8" t="s" s="2">
         <v>76</v>
@@ -2126,15 +2130,15 @@
         <v>76</v>
       </c>
       <c r="AN8" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
-    <row r="9" hidden="true">
+    <row r="9">
       <c r="A9" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
@@ -2142,31 +2146,31 @@
       </c>
       <c r="E9" s="2"/>
       <c r="F9" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G9" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H9" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I9" t="s" s="2">
         <v>76</v>
       </c>
       <c r="J9" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K9" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="L9" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="N9" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="O9" s="2"/>
       <c r="P9" t="s" s="2">
@@ -2216,19 +2220,19 @@
         <v>76</v>
       </c>
       <c r="AF9" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH9" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI9" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ9" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK9" t="s" s="2">
         <v>76</v>
@@ -2237,18 +2241,18 @@
         <v>76</v>
       </c>
       <c r="AM9" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="AN9" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" hidden="true">
       <c r="A10" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" t="s" s="2">
@@ -2259,7 +2263,7 @@
         <v>77</v>
       </c>
       <c r="G10" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H10" t="s" s="2">
         <v>76</v>
@@ -2268,19 +2272,19 @@
         <v>76</v>
       </c>
       <c r="J10" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K10" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L10" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="N10" t="s" s="2">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O10" s="2"/>
       <c r="P10" t="s" s="2">
@@ -2330,19 +2334,19 @@
         <v>76</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="AG10" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH10" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI10" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="AJ10" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK10" t="s" s="2">
         <v>76</v>
@@ -2359,10 +2363,10 @@
     </row>
     <row r="11" hidden="true">
       <c r="A11" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -2382,19 +2386,19 @@
         <v>76</v>
       </c>
       <c r="J11" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K11" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L11" t="s" s="2">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="M11" t="s" s="2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="N11" t="s" s="2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O11" s="2"/>
       <c r="P11" t="s" s="2">
@@ -2444,7 +2448,7 @@
         <v>76</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="AG11" t="s" s="2">
         <v>77</v>
@@ -2456,7 +2460,7 @@
         <v>76</v>
       </c>
       <c r="AJ11" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK11" t="s" s="2">
         <v>76</v>
@@ -2473,10 +2477,10 @@
     </row>
     <row r="12" hidden="true">
       <c r="A12" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -2487,7 +2491,7 @@
         <v>77</v>
       </c>
       <c r="G12" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H12" t="s" s="2">
         <v>76</v>
@@ -2499,13 +2503,13 @@
         <v>76</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
@@ -2556,13 +2560,13 @@
         <v>76</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH12" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI12" t="s" s="2">
         <v>76</v>
@@ -2574,7 +2578,7 @@
         <v>76</v>
       </c>
       <c r="AL12" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM12" t="s" s="2">
         <v>76</v>
@@ -2585,14 +2589,14 @@
     </row>
     <row r="13" hidden="true">
       <c r="A13" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" t="s" s="2">
@@ -2611,16 +2615,16 @@
         <v>76</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="N13" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
@@ -2670,7 +2674,7 @@
         <v>76</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>77</v>
@@ -2682,13 +2686,13 @@
         <v>76</v>
       </c>
       <c r="AJ13" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK13" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL13" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM13" t="s" s="2">
         <v>76</v>
@@ -2699,14 +2703,14 @@
     </row>
     <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" t="s" s="2">
@@ -2719,25 +2723,25 @@
         <v>76</v>
       </c>
       <c r="I14" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J14" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="N14" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O14" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="P14" t="s" s="2">
         <v>76</v>
@@ -2786,7 +2790,7 @@
         <v>76</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>77</v>
@@ -2798,13 +2802,13 @@
         <v>76</v>
       </c>
       <c r="AJ14" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK14" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL14" t="s" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AM14" t="s" s="2">
         <v>76</v>
@@ -2815,10 +2819,10 @@
     </row>
     <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
@@ -2826,10 +2830,10 @@
       </c>
       <c r="E15" s="2"/>
       <c r="F15" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G15" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H15" t="s" s="2">
         <v>76</v>
@@ -2838,16 +2842,16 @@
         <v>76</v>
       </c>
       <c r="J15" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -2898,19 +2902,19 @@
         <v>76</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="AG15" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AH15" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI15" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ15" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK15" t="s" s="2">
         <v>76</v>
@@ -2927,10 +2931,10 @@
     </row>
     <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -2938,10 +2942,10 @@
       </c>
       <c r="E16" s="2"/>
       <c r="F16" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G16" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H16" t="s" s="2">
         <v>76</v>
@@ -2950,16 +2954,16 @@
         <v>76</v>
       </c>
       <c r="J16" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
@@ -3010,19 +3014,19 @@
         <v>76</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG16" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AH16" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI16" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ16" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK16" t="s" s="2">
         <v>76</v>
@@ -3037,12 +3041,12 @@
         <v>76</v>
       </c>
     </row>
-    <row r="17" hidden="true">
+    <row r="17">
       <c r="A17" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -3056,22 +3060,22 @@
         <v>78</v>
       </c>
       <c r="H17" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I17" t="s" s="2">
         <v>76</v>
       </c>
       <c r="J17" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -3122,7 +3126,7 @@
         <v>76</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>77</v>
@@ -3134,7 +3138,7 @@
         <v>76</v>
       </c>
       <c r="AJ17" t="s" s="2">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AK17" t="s" s="2">
         <v>76</v>
@@ -3151,10 +3155,10 @@
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -3165,7 +3169,7 @@
         <v>77</v>
       </c>
       <c r="G18" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H18" t="s" s="2">
         <v>76</v>
@@ -3177,13 +3181,13 @@
         <v>76</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
@@ -3234,13 +3238,13 @@
         <v>76</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH18" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI18" t="s" s="2">
         <v>76</v>
@@ -3252,7 +3256,7 @@
         <v>76</v>
       </c>
       <c r="AL18" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM18" t="s" s="2">
         <v>76</v>
@@ -3263,14 +3267,14 @@
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
@@ -3289,16 +3293,16 @@
         <v>76</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="N19" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O19" s="2"/>
       <c r="P19" t="s" s="2">
@@ -3348,7 +3352,7 @@
         <v>76</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>77</v>
@@ -3360,13 +3364,13 @@
         <v>76</v>
       </c>
       <c r="AJ19" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK19" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL19" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM19" t="s" s="2">
         <v>76</v>
@@ -3377,14 +3381,14 @@
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" t="s" s="2">
@@ -3397,25 +3401,25 @@
         <v>76</v>
       </c>
       <c r="I20" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J20" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="N20" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O20" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="P20" t="s" s="2">
         <v>76</v>
@@ -3464,7 +3468,7 @@
         <v>76</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>77</v>
@@ -3476,13 +3480,13 @@
         <v>76</v>
       </c>
       <c r="AJ20" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK20" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL20" t="s" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AM20" t="s" s="2">
         <v>76</v>
@@ -3493,10 +3497,10 @@
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3516,16 +3520,16 @@
         <v>76</v>
       </c>
       <c r="J21" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K21" t="s" s="2">
         <v>79</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -3576,7 +3580,7 @@
         <v>76</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>77</v>
@@ -3588,7 +3592,7 @@
         <v>76</v>
       </c>
       <c r="AJ21" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK21" t="s" s="2">
         <v>76</v>
@@ -3605,10 +3609,10 @@
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3619,7 +3623,7 @@
         <v>77</v>
       </c>
       <c r="G22" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H22" t="s" s="2">
         <v>76</v>
@@ -3628,19 +3632,19 @@
         <v>76</v>
       </c>
       <c r="J22" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="N22" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="O22" s="2"/>
       <c r="P22" t="s" s="2">
@@ -3690,19 +3694,19 @@
         <v>76</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH22" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI22" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ22" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK22" t="s" s="2">
         <v>76</v>
@@ -3717,12 +3721,12 @@
         <v>76</v>
       </c>
     </row>
-    <row r="23" hidden="true">
+    <row r="23">
       <c r="A23" t="s" s="2">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3733,25 +3737,25 @@
         <v>77</v>
       </c>
       <c r="G23" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H23" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I23" t="s" s="2">
         <v>76</v>
       </c>
       <c r="J23" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
@@ -3802,13 +3806,13 @@
         <v>76</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH23" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI23" t="s" s="2">
         <v>76</v>
@@ -3831,10 +3835,10 @@
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3845,7 +3849,7 @@
         <v>77</v>
       </c>
       <c r="G24" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H24" t="s" s="2">
         <v>76</v>
@@ -3854,16 +3858,16 @@
         <v>76</v>
       </c>
       <c r="J24" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -3914,19 +3918,19 @@
         <v>76</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH24" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI24" t="s" s="2">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AJ24" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK24" t="s" s="2">
         <v>76</v>
@@ -3943,10 +3947,10 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -3957,7 +3961,7 @@
         <v>77</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>76</v>
@@ -3969,13 +3973,13 @@
         <v>76</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -4026,13 +4030,13 @@
         <v>76</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH25" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI25" t="s" s="2">
         <v>76</v>
@@ -4044,7 +4048,7 @@
         <v>76</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM25" t="s" s="2">
         <v>76</v>
@@ -4055,14 +4059,14 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
@@ -4081,16 +4085,16 @@
         <v>76</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
@@ -4140,7 +4144,7 @@
         <v>76</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>77</v>
@@ -4152,13 +4156,13 @@
         <v>76</v>
       </c>
       <c r="AJ26" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK26" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM26" t="s" s="2">
         <v>76</v>
@@ -4169,14 +4173,14 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
@@ -4189,25 +4193,25 @@
         <v>76</v>
       </c>
       <c r="I27" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J27" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="N27" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O27" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="P27" t="s" s="2">
         <v>76</v>
@@ -4256,7 +4260,7 @@
         <v>76</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>77</v>
@@ -4268,13 +4272,13 @@
         <v>76</v>
       </c>
       <c r="AJ27" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK27" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AM27" t="s" s="2">
         <v>76</v>
@@ -4285,10 +4289,10 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4299,7 +4303,7 @@
         <v>77</v>
       </c>
       <c r="G28" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H28" t="s" s="2">
         <v>76</v>
@@ -4308,19 +4312,19 @@
         <v>76</v>
       </c>
       <c r="J28" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="N28" t="s" s="2">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
@@ -4346,13 +4350,13 @@
         <v>76</v>
       </c>
       <c r="X28" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Y28" t="s" s="2">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="Z28" t="s" s="2">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AA28" t="s" s="2">
         <v>76</v>
@@ -4370,19 +4374,19 @@
         <v>76</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH28" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI28" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ28" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK28" t="s" s="2">
         <v>76</v>
@@ -4399,10 +4403,10 @@
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4413,7 +4417,7 @@
         <v>77</v>
       </c>
       <c r="G29" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H29" t="s" s="2">
         <v>76</v>
@@ -4422,19 +4426,19 @@
         <v>76</v>
       </c>
       <c r="J29" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
@@ -4484,19 +4488,19 @@
         <v>76</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH29" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI29" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ29" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK29" t="s" s="2">
         <v>76</v>
@@ -4513,10 +4517,10 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4527,7 +4531,7 @@
         <v>77</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H30" t="s" s="2">
         <v>76</v>
@@ -4536,16 +4540,16 @@
         <v>76</v>
       </c>
       <c r="J30" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
@@ -4596,19 +4600,19 @@
         <v>76</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH30" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI30" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ30" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK30" t="s" s="2">
         <v>76</v>
@@ -4625,10 +4629,10 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -4639,7 +4643,7 @@
         <v>77</v>
       </c>
       <c r="G31" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H31" t="s" s="2">
         <v>76</v>
@@ -4651,13 +4655,13 @@
         <v>76</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -4708,13 +4712,13 @@
         <v>76</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH31" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI31" t="s" s="2">
         <v>76</v>
@@ -4726,7 +4730,7 @@
         <v>76</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM31" t="s" s="2">
         <v>76</v>
@@ -4737,14 +4741,14 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
@@ -4763,16 +4767,16 @@
         <v>76</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="N32" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
@@ -4822,7 +4826,7 @@
         <v>76</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>77</v>
@@ -4834,13 +4838,13 @@
         <v>76</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK32" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL32" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM32" t="s" s="2">
         <v>76</v>
@@ -4851,14 +4855,14 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
@@ -4871,25 +4875,25 @@
         <v>76</v>
       </c>
       <c r="I33" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J33" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O33" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="P33" t="s" s="2">
         <v>76</v>
@@ -4938,7 +4942,7 @@
         <v>76</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>77</v>
@@ -4950,13 +4954,13 @@
         <v>76</v>
       </c>
       <c r="AJ33" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK33" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL33" t="s" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AM33" t="s" s="2">
         <v>76</v>
@@ -4967,10 +4971,10 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -4978,10 +4982,10 @@
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G34" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H34" t="s" s="2">
         <v>76</v>
@@ -4990,16 +4994,16 @@
         <v>76</v>
       </c>
       <c r="J34" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -5026,13 +5030,13 @@
         <v>76</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Y34" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="Z34" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>76</v>
@@ -5050,19 +5054,19 @@
         <v>76</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="AG34" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AH34" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI34" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK34" t="s" s="2">
         <v>76</v>
@@ -5079,10 +5083,10 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5090,10 +5094,10 @@
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G35" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H35" t="s" s="2">
         <v>76</v>
@@ -5102,19 +5106,19 @@
         <v>76</v>
       </c>
       <c r="J35" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="N35" t="s" s="2">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
@@ -5164,19 +5168,19 @@
         <v>76</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="AG35" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AH35" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI35" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ35" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK35" t="s" s="2">
         <v>76</v>
@@ -5193,10 +5197,10 @@
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5207,7 +5211,7 @@
         <v>77</v>
       </c>
       <c r="G36" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H36" t="s" s="2">
         <v>76</v>
@@ -5216,16 +5220,16 @@
         <v>76</v>
       </c>
       <c r="J36" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -5276,19 +5280,19 @@
         <v>76</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH36" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI36" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ36" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK36" t="s" s="2">
         <v>76</v>
@@ -5305,10 +5309,10 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5319,7 +5323,7 @@
         <v>77</v>
       </c>
       <c r="G37" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H37" t="s" s="2">
         <v>76</v>
@@ -5328,16 +5332,16 @@
         <v>76</v>
       </c>
       <c r="J37" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
@@ -5388,19 +5392,19 @@
         <v>76</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH37" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI37" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ37" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK37" t="s" s="2">
         <v>76</v>
@@ -5417,10 +5421,10 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5431,7 +5435,7 @@
         <v>77</v>
       </c>
       <c r="G38" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H38" t="s" s="2">
         <v>76</v>
@@ -5440,16 +5444,16 @@
         <v>76</v>
       </c>
       <c r="J38" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -5500,19 +5504,19 @@
         <v>76</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH38" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI38" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ38" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK38" t="s" s="2">
         <v>76</v>
@@ -5529,10 +5533,10 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5543,7 +5547,7 @@
         <v>77</v>
       </c>
       <c r="G39" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H39" t="s" s="2">
         <v>76</v>
@@ -5552,16 +5556,16 @@
         <v>76</v>
       </c>
       <c r="J39" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -5612,19 +5616,19 @@
         <v>76</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH39" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI39" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ39" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK39" t="s" s="2">
         <v>76</v>
@@ -5641,10 +5645,10 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5655,7 +5659,7 @@
         <v>77</v>
       </c>
       <c r="G40" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H40" t="s" s="2">
         <v>76</v>
@@ -5664,16 +5668,16 @@
         <v>76</v>
       </c>
       <c r="J40" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -5724,19 +5728,19 @@
         <v>76</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH40" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI40" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="AJ40" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK40" t="s" s="2">
         <v>76</v>
@@ -5753,10 +5757,10 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -5767,7 +5771,7 @@
         <v>77</v>
       </c>
       <c r="G41" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H41" t="s" s="2">
         <v>76</v>
@@ -5779,13 +5783,13 @@
         <v>76</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -5836,13 +5840,13 @@
         <v>76</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH41" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI41" t="s" s="2">
         <v>76</v>
@@ -5854,7 +5858,7 @@
         <v>76</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM41" t="s" s="2">
         <v>76</v>
@@ -5865,14 +5869,14 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
@@ -5891,16 +5895,16 @@
         <v>76</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="N42" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O42" s="2"/>
       <c r="P42" t="s" s="2">
@@ -5950,7 +5954,7 @@
         <v>76</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>77</v>
@@ -5962,13 +5966,13 @@
         <v>76</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK42" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM42" t="s" s="2">
         <v>76</v>
@@ -5979,14 +5983,14 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
@@ -5999,25 +6003,25 @@
         <v>76</v>
       </c>
       <c r="I43" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J43" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="N43" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O43" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="P43" t="s" s="2">
         <v>76</v>
@@ -6066,7 +6070,7 @@
         <v>76</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>77</v>
@@ -6078,13 +6082,13 @@
         <v>76</v>
       </c>
       <c r="AJ43" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK43" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL43" t="s" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AM43" t="s" s="2">
         <v>76</v>
@@ -6095,10 +6099,10 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6106,10 +6110,10 @@
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G44" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H44" t="s" s="2">
         <v>76</v>
@@ -6118,16 +6122,16 @@
         <v>76</v>
       </c>
       <c r="J44" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
@@ -6178,19 +6182,19 @@
         <v>76</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AG44" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AH44" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI44" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ44" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK44" t="s" s="2">
         <v>76</v>
@@ -6207,10 +6211,10 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6221,7 +6225,7 @@
         <v>77</v>
       </c>
       <c r="G45" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H45" t="s" s="2">
         <v>76</v>
@@ -6230,16 +6234,16 @@
         <v>76</v>
       </c>
       <c r="J45" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
@@ -6290,19 +6294,19 @@
         <v>76</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH45" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI45" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ45" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK45" t="s" s="2">
         <v>76</v>
@@ -6319,10 +6323,10 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6333,7 +6337,7 @@
         <v>77</v>
       </c>
       <c r="G46" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H46" t="s" s="2">
         <v>76</v>
@@ -6342,19 +6346,19 @@
         <v>76</v>
       </c>
       <c r="J46" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="N46" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
@@ -6404,19 +6408,19 @@
         <v>76</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH46" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI46" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ46" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK46" t="s" s="2">
         <v>76</v>
@@ -6433,10 +6437,10 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -6447,7 +6451,7 @@
         <v>77</v>
       </c>
       <c r="G47" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H47" t="s" s="2">
         <v>76</v>
@@ -6456,19 +6460,19 @@
         <v>76</v>
       </c>
       <c r="J47" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="N47" t="s" s="2">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
@@ -6518,19 +6522,19 @@
         <v>76</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH47" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI47" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ47" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK47" t="s" s="2">
         <v>76</v>
@@ -6547,10 +6551,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -6561,7 +6565,7 @@
         <v>77</v>
       </c>
       <c r="G48" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H48" t="s" s="2">
         <v>76</v>
@@ -6570,19 +6574,19 @@
         <v>76</v>
       </c>
       <c r="J48" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="N48" t="s" s="2">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="O48" s="2"/>
       <c r="P48" t="s" s="2">
@@ -6632,13 +6636,13 @@
         <v>76</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH48" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI48" t="s" s="2">
         <v>76</v>
@@ -6661,10 +6665,10 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -6675,7 +6679,7 @@
         <v>77</v>
       </c>
       <c r="G49" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H49" t="s" s="2">
         <v>76</v>
@@ -6684,22 +6688,22 @@
         <v>76</v>
       </c>
       <c r="J49" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="N49" t="s" s="2">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="O49" t="s" s="2">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="P49" t="s" s="2">
         <v>76</v>
@@ -6748,19 +6752,19 @@
         <v>76</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH49" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI49" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ49" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK49" t="s" s="2">
         <v>76</v>
@@ -6777,12 +6781,12 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AN49">
-    <filterColumn colId="6">
+    <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
       </customFilters>
     </filterColumn>
-    <filterColumn colId="26">
+    <filterColumn colId="27">
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
chore: publish hospitalnotification IG 3.0.2 (#64)
Co-authored-by: tmsMedcom <tmsMedcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ig/hospitalnotification/StructureDefinition-medcom-hospitalNotification-message.xlsx
+++ b/ig/hospitalnotification/StructureDefinition-medcom-hospitalNotification-message.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1788" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1788" uniqueCount="268">
   <si>
     <t>Property</t>
   </si>
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>3.0.1</t>
+    <t>3.0.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-03-02T09:56:15+01:00</t>
+    <t>2026-02-10T12:55:02+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -69,7 +69,7 @@
     <t>Contact</t>
   </si>
   <si>
-    <t>No display for ContactDetail</t>
+    <t>MedCom (http://www.medcom.dk)</t>
   </si>
   <si>
     <t>Jurisdiction</t>
@@ -263,6 +263,10 @@
   </si>
   <si>
     <t>A container for a collection of resources.</t>
+  </si>
+  <si>
+    <t>bdl-1:total only when a search or history {total.empty() or (type = 'searchset') or (type = 'history')}
+bdl-2:entry.search only when a search {entry.search.empty() or (type = 'searchset')}bdl-3:entry.request mandatory for batch/transaction/history, otherwise prohibited {entry.all(request.exists() = (%resource.type = 'batch' or %resource.type = 'transaction' or %resource.type = 'history'))}bdl-4:entry.response mandatory for batch-response/transaction-response/history, otherwise prohibited {entry.all(response.exists() = (%resource.type = 'batch-response' or %resource.type = 'transaction-response' or %resource.type = 'history'))}bdl-7:FullUrl must be unique in a bundle, or else entries with the same fullUrl must have different meta.versionId (except in history bundles) {(type = 'history') or entry.where(fullUrl.exists()).select(fullUrl&amp;resource.meta.versionId).isDistinct()}bdl-9:A document must have an identifier with a system and a value {type = 'document' implies (identifier.system.exists() and identifier.value.exists())}bdl-10:A document must have a date {type = 'document' implies (timestamp.hasValue())}bdl-11:A document must have a Composition as the first resource {type = 'document' implies entry.first().resource.is(Composition)}bdl-12:A message must have a MessageHeader as the first resource {type = 'message' implies entry.first().resource.is(MessageHeader)}medcom-messaging-1:The MessageHeader resource shall conform to medcom-messaging-messageHeader profile {entry.ofType(MessageHeader).all(resource.conformsTo('http://medcomfhir.dk/fhir/messaging/StructureDefinition/medcom-messaging-messageHeader'))}medcom-messaging-2:There shall be at least one Provenance resource in a MedCom message {entry.resource.ofType(Provenance).exists()}medcom-messaging-3:All Provenance resources shall conform to medcom-core-provenance profile {entry.ofType(Provenance).all(resource.conformsTo('http://medcomfhir.dk/fhir/messaging/StructureDefinition/medcom-messaging-provenance'))}medcom-hospitalNotification-1:The message header shall conform to medcom-hospitalNotification-messageHeader profile {entry.ofType(MessageHeader).all(resource.conformsTo('http://medcomfhir.dk/fhir/hospitalnotification/StructureDefinition/medcom-hospitalNotification-messageHeader'))}medcom-hospitalNotification-2:Entry shall contain exactly one patient resource {entry.where(resource.is(Patient)).count() = 1}medcom-hospitalNotification-3:All provenance resources shall contain activities from medcom-hospitalNotification-messageActivities valueset {entry.ofType(Provenance).all(resource.activity.memberOf('http://medcomfhir.dk/fhir/dk-medcom-terminology/ValueSet/medcom-hospitalNotification-messageActivities'))}medcom-hospitalNotification-4:The system of Patient.identifier shall be 'urn:oid:1.2.208.176.1.2', which represents an official Danish CPR-number {entry.resource.ofType(Patient).identifier.system = 'urn:oid:1.2.208.176.1.2'}medcom-hospitalNotification-5:The receiver of a HospitalNotification shall always be a primary receiver. {Bundle.entry.resource.ofType(MessageHeader).destination.extension.value.code = 'primary'}</t>
   </si>
   <si>
     <t>N/A</t>
@@ -976,10 +980,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyBorder="true" applyFill="true" applyFont="true">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyBorder="true" applyFill="true" applyAlignment="true" applyFont="true">
       <alignment vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="true" applyAlignment="true">
       <alignment vertical="top" wrapText="true"/>
     </xf>
   </cellXfs>
@@ -1172,17 +1176,17 @@
   <dimension ref="A1:AN49"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="38.1796875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="38.1796875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.1328125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="4" max="4" width="20.859375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="5" max="5" width="5.90234375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="4.69921875" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="5.07421875" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="14.625" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="11.98828125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="33.44140625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="33.44140625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="4" max="4" width="18.19140625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="4.65625" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="17.203125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="15.140625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -1191,26 +1195,26 @@
     <col min="17" max="17" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="18" max="18" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="19" max="19" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" width="8.84375" customWidth="true" bestFit="true"/>
-    <col min="21" max="21" width="15.71484375" customWidth="true" bestFit="true"/>
-    <col min="22" max="22" width="16.08984375" customWidth="true" bestFit="true"/>
-    <col min="23" max="23" width="17.078125" customWidth="true" bestFit="true"/>
-    <col min="24" max="24" width="16.3125" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="163.2734375" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="49.55078125" customWidth="true" bestFit="true"/>
-    <col min="27" max="27" width="5.69140625" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="19.73046875" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" width="17.8203125" customWidth="true" bestFit="true"/>
-    <col min="30" max="30" width="14.98828125" customWidth="true" bestFit="true"/>
-    <col min="31" max="31" width="12.3046875" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="34.5859375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="33" max="33" width="9.5" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="34" max="34" width="9.87890625" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" width="8.53515625" customWidth="true" bestFit="true"/>
+    <col min="21" max="21" width="14.72265625" customWidth="true" bestFit="true"/>
+    <col min="22" max="22" width="15.13671875" customWidth="true" bestFit="true"/>
+    <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
+    <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="144.1953125" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="42.01953125" customWidth="true" bestFit="true"/>
+    <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
+    <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
+    <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="29.98828125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
-    <col min="37" max="37" width="25.01171875" customWidth="true" bestFit="true"/>
-    <col min="38" max="38" width="22.67578125" customWidth="true" bestFit="true"/>
-    <col min="39" max="39" width="41.43359375" customWidth="true" bestFit="true"/>
-    <col min="40" max="40" width="32.84375" customWidth="true" bestFit="true"/>
+    <col min="37" max="37" width="24.1328125" customWidth="true" bestFit="true"/>
+    <col min="38" max="38" width="21.4140625" customWidth="true" bestFit="true"/>
+    <col min="39" max="39" width="36.84375" customWidth="true" bestFit="true"/>
+    <col min="40" max="40" width="31.65234375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1432,27 +1436,27 @@
         <v>76</v>
       </c>
       <c r="AJ2" t="s" s="2">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="AK2" t="s" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AL2" t="s" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AM2" t="s" s="2">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AN2" t="s" s="2">
         <v>76</v>
       </c>
     </row>
-    <row r="3" hidden="true">
+    <row r="3">
       <c r="A3" t="s" s="2">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" t="s" s="2">
@@ -1460,31 +1464,31 @@
       </c>
       <c r="E3" s="2"/>
       <c r="F3" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G3" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H3" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I3" t="s" s="2">
         <v>76</v>
       </c>
       <c r="J3" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K3" t="s" s="2">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L3" t="s" s="2">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="M3" t="s" s="2">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="N3" t="s" s="2">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O3" s="2"/>
       <c r="P3" t="s" s="2">
@@ -1534,13 +1538,13 @@
         <v>76</v>
       </c>
       <c r="AF3" t="s" s="2">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="AG3" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH3" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI3" t="s" s="2">
         <v>76</v>
@@ -1563,10 +1567,10 @@
     </row>
     <row r="4" hidden="true">
       <c r="A4" t="s" s="2">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" t="s" s="2">
@@ -1577,7 +1581,7 @@
         <v>77</v>
       </c>
       <c r="G4" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H4" t="s" s="2">
         <v>76</v>
@@ -1586,16 +1590,16 @@
         <v>76</v>
       </c>
       <c r="J4" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K4" t="s" s="2">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L4" t="s" s="2">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="M4" t="s" s="2">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
@@ -1646,19 +1650,19 @@
         <v>76</v>
       </c>
       <c r="AF4" t="s" s="2">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AG4" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH4" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI4" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ4" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK4" t="s" s="2">
         <v>76</v>
@@ -1675,10 +1679,10 @@
     </row>
     <row r="5" hidden="true">
       <c r="A5" t="s" s="2">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" t="s" s="2">
@@ -1689,28 +1693,28 @@
         <v>77</v>
       </c>
       <c r="G5" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H5" t="s" s="2">
         <v>76</v>
       </c>
       <c r="I5" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J5" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K5" t="s" s="2">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L5" t="s" s="2">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M5" t="s" s="2">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="N5" t="s" s="2">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="O5" s="2"/>
       <c r="P5" t="s" s="2">
@@ -1760,19 +1764,19 @@
         <v>76</v>
       </c>
       <c r="AF5" t="s" s="2">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AG5" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH5" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI5" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ5" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK5" t="s" s="2">
         <v>76</v>
@@ -1789,10 +1793,10 @@
     </row>
     <row r="6" hidden="true">
       <c r="A6" t="s" s="2">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" t="s" s="2">
@@ -1803,7 +1807,7 @@
         <v>77</v>
       </c>
       <c r="G6" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H6" t="s" s="2">
         <v>76</v>
@@ -1815,16 +1819,16 @@
         <v>76</v>
       </c>
       <c r="K6" t="s" s="2">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L6" t="s" s="2">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M6" t="s" s="2">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N6" t="s" s="2">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="O6" s="2"/>
       <c r="P6" t="s" s="2">
@@ -1850,13 +1854,13 @@
         <v>76</v>
       </c>
       <c r="X6" t="s" s="2">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="Y6" t="s" s="2">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="Z6" t="s" s="2">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="AA6" t="s" s="2">
         <v>76</v>
@@ -1874,19 +1878,19 @@
         <v>76</v>
       </c>
       <c r="AF6" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AG6" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH6" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI6" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ6" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK6" t="s" s="2">
         <v>76</v>
@@ -1903,10 +1907,10 @@
     </row>
     <row r="7" hidden="true">
       <c r="A7" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" t="s" s="2">
@@ -1917,7 +1921,7 @@
         <v>77</v>
       </c>
       <c r="G7" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H7" t="s" s="2">
         <v>76</v>
@@ -1926,19 +1930,19 @@
         <v>76</v>
       </c>
       <c r="J7" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K7" t="s" s="2">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="L7" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="M7" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="N7" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="O7" s="2"/>
       <c r="P7" t="s" s="2">
@@ -1988,19 +1992,19 @@
         <v>76</v>
       </c>
       <c r="AF7" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH7" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI7" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ7" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK7" t="s" s="2">
         <v>76</v>
@@ -2009,18 +2013,18 @@
         <v>76</v>
       </c>
       <c r="AM7" t="s" s="2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AN7" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
-    <row r="8" hidden="true">
+    <row r="8">
       <c r="A8" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -2028,31 +2032,31 @@
       </c>
       <c r="E8" s="2"/>
       <c r="F8" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G8" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H8" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I8" t="s" s="2">
         <v>76</v>
       </c>
       <c r="J8" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K8" t="s" s="2">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L8" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M8" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N8" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="O8" s="2"/>
       <c r="P8" t="s" s="2">
@@ -2063,7 +2067,7 @@
         <v>76</v>
       </c>
       <c r="S8" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="T8" t="s" s="2">
         <v>76</v>
@@ -2078,13 +2082,13 @@
         <v>76</v>
       </c>
       <c r="X8" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Y8" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Z8" t="s" s="2">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AA8" t="s" s="2">
         <v>76</v>
@@ -2102,19 +2106,19 @@
         <v>76</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AG8" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AH8" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI8" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ8" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK8" t="s" s="2">
         <v>76</v>
@@ -2126,15 +2130,15 @@
         <v>76</v>
       </c>
       <c r="AN8" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
-    <row r="9" hidden="true">
+    <row r="9">
       <c r="A9" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
@@ -2142,31 +2146,31 @@
       </c>
       <c r="E9" s="2"/>
       <c r="F9" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G9" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H9" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I9" t="s" s="2">
         <v>76</v>
       </c>
       <c r="J9" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K9" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="L9" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="N9" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="O9" s="2"/>
       <c r="P9" t="s" s="2">
@@ -2216,19 +2220,19 @@
         <v>76</v>
       </c>
       <c r="AF9" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH9" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI9" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ9" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK9" t="s" s="2">
         <v>76</v>
@@ -2237,18 +2241,18 @@
         <v>76</v>
       </c>
       <c r="AM9" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="AN9" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" hidden="true">
       <c r="A10" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" t="s" s="2">
@@ -2259,7 +2263,7 @@
         <v>77</v>
       </c>
       <c r="G10" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H10" t="s" s="2">
         <v>76</v>
@@ -2268,19 +2272,19 @@
         <v>76</v>
       </c>
       <c r="J10" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K10" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L10" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="N10" t="s" s="2">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O10" s="2"/>
       <c r="P10" t="s" s="2">
@@ -2330,19 +2334,19 @@
         <v>76</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="AG10" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH10" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI10" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="AJ10" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK10" t="s" s="2">
         <v>76</v>
@@ -2359,10 +2363,10 @@
     </row>
     <row r="11" hidden="true">
       <c r="A11" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -2382,19 +2386,19 @@
         <v>76</v>
       </c>
       <c r="J11" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K11" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L11" t="s" s="2">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="M11" t="s" s="2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="N11" t="s" s="2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O11" s="2"/>
       <c r="P11" t="s" s="2">
@@ -2444,7 +2448,7 @@
         <v>76</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="AG11" t="s" s="2">
         <v>77</v>
@@ -2456,7 +2460,7 @@
         <v>76</v>
       </c>
       <c r="AJ11" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK11" t="s" s="2">
         <v>76</v>
@@ -2473,10 +2477,10 @@
     </row>
     <row r="12" hidden="true">
       <c r="A12" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -2487,7 +2491,7 @@
         <v>77</v>
       </c>
       <c r="G12" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H12" t="s" s="2">
         <v>76</v>
@@ -2499,13 +2503,13 @@
         <v>76</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
@@ -2556,13 +2560,13 @@
         <v>76</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH12" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI12" t="s" s="2">
         <v>76</v>
@@ -2574,7 +2578,7 @@
         <v>76</v>
       </c>
       <c r="AL12" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM12" t="s" s="2">
         <v>76</v>
@@ -2585,14 +2589,14 @@
     </row>
     <row r="13" hidden="true">
       <c r="A13" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" t="s" s="2">
@@ -2611,16 +2615,16 @@
         <v>76</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="N13" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
@@ -2670,7 +2674,7 @@
         <v>76</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>77</v>
@@ -2682,13 +2686,13 @@
         <v>76</v>
       </c>
       <c r="AJ13" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK13" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL13" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM13" t="s" s="2">
         <v>76</v>
@@ -2699,14 +2703,14 @@
     </row>
     <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" t="s" s="2">
@@ -2719,25 +2723,25 @@
         <v>76</v>
       </c>
       <c r="I14" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J14" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="N14" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O14" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="P14" t="s" s="2">
         <v>76</v>
@@ -2786,7 +2790,7 @@
         <v>76</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>77</v>
@@ -2798,13 +2802,13 @@
         <v>76</v>
       </c>
       <c r="AJ14" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK14" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL14" t="s" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AM14" t="s" s="2">
         <v>76</v>
@@ -2815,10 +2819,10 @@
     </row>
     <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
@@ -2826,10 +2830,10 @@
       </c>
       <c r="E15" s="2"/>
       <c r="F15" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G15" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H15" t="s" s="2">
         <v>76</v>
@@ -2838,16 +2842,16 @@
         <v>76</v>
       </c>
       <c r="J15" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -2898,19 +2902,19 @@
         <v>76</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="AG15" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AH15" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI15" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ15" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK15" t="s" s="2">
         <v>76</v>
@@ -2927,10 +2931,10 @@
     </row>
     <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -2938,10 +2942,10 @@
       </c>
       <c r="E16" s="2"/>
       <c r="F16" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G16" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H16" t="s" s="2">
         <v>76</v>
@@ -2950,16 +2954,16 @@
         <v>76</v>
       </c>
       <c r="J16" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
@@ -3010,19 +3014,19 @@
         <v>76</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG16" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AH16" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI16" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ16" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK16" t="s" s="2">
         <v>76</v>
@@ -3037,12 +3041,12 @@
         <v>76</v>
       </c>
     </row>
-    <row r="17" hidden="true">
+    <row r="17">
       <c r="A17" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -3056,22 +3060,22 @@
         <v>78</v>
       </c>
       <c r="H17" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I17" t="s" s="2">
         <v>76</v>
       </c>
       <c r="J17" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -3122,7 +3126,7 @@
         <v>76</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>77</v>
@@ -3134,7 +3138,7 @@
         <v>76</v>
       </c>
       <c r="AJ17" t="s" s="2">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AK17" t="s" s="2">
         <v>76</v>
@@ -3151,10 +3155,10 @@
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -3165,7 +3169,7 @@
         <v>77</v>
       </c>
       <c r="G18" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H18" t="s" s="2">
         <v>76</v>
@@ -3177,13 +3181,13 @@
         <v>76</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
@@ -3234,13 +3238,13 @@
         <v>76</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH18" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI18" t="s" s="2">
         <v>76</v>
@@ -3252,7 +3256,7 @@
         <v>76</v>
       </c>
       <c r="AL18" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM18" t="s" s="2">
         <v>76</v>
@@ -3263,14 +3267,14 @@
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
@@ -3289,16 +3293,16 @@
         <v>76</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="N19" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O19" s="2"/>
       <c r="P19" t="s" s="2">
@@ -3348,7 +3352,7 @@
         <v>76</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>77</v>
@@ -3360,13 +3364,13 @@
         <v>76</v>
       </c>
       <c r="AJ19" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK19" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL19" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM19" t="s" s="2">
         <v>76</v>
@@ -3377,14 +3381,14 @@
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" t="s" s="2">
@@ -3397,25 +3401,25 @@
         <v>76</v>
       </c>
       <c r="I20" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J20" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="N20" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O20" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="P20" t="s" s="2">
         <v>76</v>
@@ -3464,7 +3468,7 @@
         <v>76</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>77</v>
@@ -3476,13 +3480,13 @@
         <v>76</v>
       </c>
       <c r="AJ20" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK20" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL20" t="s" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AM20" t="s" s="2">
         <v>76</v>
@@ -3493,10 +3497,10 @@
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3516,16 +3520,16 @@
         <v>76</v>
       </c>
       <c r="J21" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K21" t="s" s="2">
         <v>79</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -3576,7 +3580,7 @@
         <v>76</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>77</v>
@@ -3588,7 +3592,7 @@
         <v>76</v>
       </c>
       <c r="AJ21" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK21" t="s" s="2">
         <v>76</v>
@@ -3605,10 +3609,10 @@
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3619,7 +3623,7 @@
         <v>77</v>
       </c>
       <c r="G22" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H22" t="s" s="2">
         <v>76</v>
@@ -3628,19 +3632,19 @@
         <v>76</v>
       </c>
       <c r="J22" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="N22" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="O22" s="2"/>
       <c r="P22" t="s" s="2">
@@ -3690,19 +3694,19 @@
         <v>76</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH22" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI22" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ22" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK22" t="s" s="2">
         <v>76</v>
@@ -3717,12 +3721,12 @@
         <v>76</v>
       </c>
     </row>
-    <row r="23" hidden="true">
+    <row r="23">
       <c r="A23" t="s" s="2">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3733,25 +3737,25 @@
         <v>77</v>
       </c>
       <c r="G23" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H23" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I23" t="s" s="2">
         <v>76</v>
       </c>
       <c r="J23" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
@@ -3802,13 +3806,13 @@
         <v>76</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH23" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI23" t="s" s="2">
         <v>76</v>
@@ -3831,10 +3835,10 @@
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3845,7 +3849,7 @@
         <v>77</v>
       </c>
       <c r="G24" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H24" t="s" s="2">
         <v>76</v>
@@ -3854,16 +3858,16 @@
         <v>76</v>
       </c>
       <c r="J24" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -3914,19 +3918,19 @@
         <v>76</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH24" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI24" t="s" s="2">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AJ24" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK24" t="s" s="2">
         <v>76</v>
@@ -3943,10 +3947,10 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -3957,7 +3961,7 @@
         <v>77</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>76</v>
@@ -3969,13 +3973,13 @@
         <v>76</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -4026,13 +4030,13 @@
         <v>76</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH25" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI25" t="s" s="2">
         <v>76</v>
@@ -4044,7 +4048,7 @@
         <v>76</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM25" t="s" s="2">
         <v>76</v>
@@ -4055,14 +4059,14 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
@@ -4081,16 +4085,16 @@
         <v>76</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
@@ -4140,7 +4144,7 @@
         <v>76</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>77</v>
@@ -4152,13 +4156,13 @@
         <v>76</v>
       </c>
       <c r="AJ26" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK26" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM26" t="s" s="2">
         <v>76</v>
@@ -4169,14 +4173,14 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
@@ -4189,25 +4193,25 @@
         <v>76</v>
       </c>
       <c r="I27" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J27" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="N27" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O27" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="P27" t="s" s="2">
         <v>76</v>
@@ -4256,7 +4260,7 @@
         <v>76</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>77</v>
@@ -4268,13 +4272,13 @@
         <v>76</v>
       </c>
       <c r="AJ27" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK27" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AM27" t="s" s="2">
         <v>76</v>
@@ -4285,10 +4289,10 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4299,7 +4303,7 @@
         <v>77</v>
       </c>
       <c r="G28" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H28" t="s" s="2">
         <v>76</v>
@@ -4308,19 +4312,19 @@
         <v>76</v>
       </c>
       <c r="J28" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="N28" t="s" s="2">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
@@ -4346,13 +4350,13 @@
         <v>76</v>
       </c>
       <c r="X28" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Y28" t="s" s="2">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="Z28" t="s" s="2">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AA28" t="s" s="2">
         <v>76</v>
@@ -4370,19 +4374,19 @@
         <v>76</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH28" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI28" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ28" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK28" t="s" s="2">
         <v>76</v>
@@ -4399,10 +4403,10 @@
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4413,7 +4417,7 @@
         <v>77</v>
       </c>
       <c r="G29" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H29" t="s" s="2">
         <v>76</v>
@@ -4422,19 +4426,19 @@
         <v>76</v>
       </c>
       <c r="J29" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
@@ -4484,19 +4488,19 @@
         <v>76</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH29" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI29" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ29" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK29" t="s" s="2">
         <v>76</v>
@@ -4513,10 +4517,10 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4527,7 +4531,7 @@
         <v>77</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H30" t="s" s="2">
         <v>76</v>
@@ -4536,16 +4540,16 @@
         <v>76</v>
       </c>
       <c r="J30" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
@@ -4596,19 +4600,19 @@
         <v>76</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH30" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI30" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ30" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK30" t="s" s="2">
         <v>76</v>
@@ -4625,10 +4629,10 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -4639,7 +4643,7 @@
         <v>77</v>
       </c>
       <c r="G31" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H31" t="s" s="2">
         <v>76</v>
@@ -4651,13 +4655,13 @@
         <v>76</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -4708,13 +4712,13 @@
         <v>76</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH31" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI31" t="s" s="2">
         <v>76</v>
@@ -4726,7 +4730,7 @@
         <v>76</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM31" t="s" s="2">
         <v>76</v>
@@ -4737,14 +4741,14 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
@@ -4763,16 +4767,16 @@
         <v>76</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="N32" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
@@ -4822,7 +4826,7 @@
         <v>76</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>77</v>
@@ -4834,13 +4838,13 @@
         <v>76</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK32" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL32" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM32" t="s" s="2">
         <v>76</v>
@@ -4851,14 +4855,14 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
@@ -4871,25 +4875,25 @@
         <v>76</v>
       </c>
       <c r="I33" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J33" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O33" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="P33" t="s" s="2">
         <v>76</v>
@@ -4938,7 +4942,7 @@
         <v>76</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>77</v>
@@ -4950,13 +4954,13 @@
         <v>76</v>
       </c>
       <c r="AJ33" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK33" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL33" t="s" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AM33" t="s" s="2">
         <v>76</v>
@@ -4967,10 +4971,10 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -4978,10 +4982,10 @@
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G34" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H34" t="s" s="2">
         <v>76</v>
@@ -4990,16 +4994,16 @@
         <v>76</v>
       </c>
       <c r="J34" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -5026,13 +5030,13 @@
         <v>76</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Y34" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="Z34" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>76</v>
@@ -5050,19 +5054,19 @@
         <v>76</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="AG34" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AH34" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI34" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK34" t="s" s="2">
         <v>76</v>
@@ -5079,10 +5083,10 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5090,10 +5094,10 @@
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G35" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H35" t="s" s="2">
         <v>76</v>
@@ -5102,19 +5106,19 @@
         <v>76</v>
       </c>
       <c r="J35" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="N35" t="s" s="2">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
@@ -5164,19 +5168,19 @@
         <v>76</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="AG35" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AH35" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI35" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ35" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK35" t="s" s="2">
         <v>76</v>
@@ -5193,10 +5197,10 @@
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5207,7 +5211,7 @@
         <v>77</v>
       </c>
       <c r="G36" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H36" t="s" s="2">
         <v>76</v>
@@ -5216,16 +5220,16 @@
         <v>76</v>
       </c>
       <c r="J36" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -5276,19 +5280,19 @@
         <v>76</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH36" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI36" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ36" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK36" t="s" s="2">
         <v>76</v>
@@ -5305,10 +5309,10 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5319,7 +5323,7 @@
         <v>77</v>
       </c>
       <c r="G37" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H37" t="s" s="2">
         <v>76</v>
@@ -5328,16 +5332,16 @@
         <v>76</v>
       </c>
       <c r="J37" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
@@ -5388,19 +5392,19 @@
         <v>76</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH37" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI37" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ37" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK37" t="s" s="2">
         <v>76</v>
@@ -5417,10 +5421,10 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5431,7 +5435,7 @@
         <v>77</v>
       </c>
       <c r="G38" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H38" t="s" s="2">
         <v>76</v>
@@ -5440,16 +5444,16 @@
         <v>76</v>
       </c>
       <c r="J38" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -5500,19 +5504,19 @@
         <v>76</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH38" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI38" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ38" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK38" t="s" s="2">
         <v>76</v>
@@ -5529,10 +5533,10 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5543,7 +5547,7 @@
         <v>77</v>
       </c>
       <c r="G39" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H39" t="s" s="2">
         <v>76</v>
@@ -5552,16 +5556,16 @@
         <v>76</v>
       </c>
       <c r="J39" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -5612,19 +5616,19 @@
         <v>76</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH39" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI39" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ39" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK39" t="s" s="2">
         <v>76</v>
@@ -5641,10 +5645,10 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5655,7 +5659,7 @@
         <v>77</v>
       </c>
       <c r="G40" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H40" t="s" s="2">
         <v>76</v>
@@ -5664,16 +5668,16 @@
         <v>76</v>
       </c>
       <c r="J40" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -5724,19 +5728,19 @@
         <v>76</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH40" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI40" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="AJ40" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK40" t="s" s="2">
         <v>76</v>
@@ -5753,10 +5757,10 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -5767,7 +5771,7 @@
         <v>77</v>
       </c>
       <c r="G41" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H41" t="s" s="2">
         <v>76</v>
@@ -5779,13 +5783,13 @@
         <v>76</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -5836,13 +5840,13 @@
         <v>76</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH41" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI41" t="s" s="2">
         <v>76</v>
@@ -5854,7 +5858,7 @@
         <v>76</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM41" t="s" s="2">
         <v>76</v>
@@ -5865,14 +5869,14 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
@@ -5891,16 +5895,16 @@
         <v>76</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="N42" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O42" s="2"/>
       <c r="P42" t="s" s="2">
@@ -5950,7 +5954,7 @@
         <v>76</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>77</v>
@@ -5962,13 +5966,13 @@
         <v>76</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK42" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AM42" t="s" s="2">
         <v>76</v>
@@ -5979,14 +5983,14 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
@@ -5999,25 +6003,25 @@
         <v>76</v>
       </c>
       <c r="I43" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J43" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="N43" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O43" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="P43" t="s" s="2">
         <v>76</v>
@@ -6066,7 +6070,7 @@
         <v>76</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>77</v>
@@ -6078,13 +6082,13 @@
         <v>76</v>
       </c>
       <c r="AJ43" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AK43" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL43" t="s" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AM43" t="s" s="2">
         <v>76</v>
@@ -6095,10 +6099,10 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6106,10 +6110,10 @@
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G44" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H44" t="s" s="2">
         <v>76</v>
@@ -6118,16 +6122,16 @@
         <v>76</v>
       </c>
       <c r="J44" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
@@ -6178,19 +6182,19 @@
         <v>76</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AG44" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AH44" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI44" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ44" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK44" t="s" s="2">
         <v>76</v>
@@ -6207,10 +6211,10 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6221,7 +6225,7 @@
         <v>77</v>
       </c>
       <c r="G45" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H45" t="s" s="2">
         <v>76</v>
@@ -6230,16 +6234,16 @@
         <v>76</v>
       </c>
       <c r="J45" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
@@ -6290,19 +6294,19 @@
         <v>76</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH45" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI45" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ45" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK45" t="s" s="2">
         <v>76</v>
@@ -6319,10 +6323,10 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6333,7 +6337,7 @@
         <v>77</v>
       </c>
       <c r="G46" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H46" t="s" s="2">
         <v>76</v>
@@ -6342,19 +6346,19 @@
         <v>76</v>
       </c>
       <c r="J46" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="N46" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
@@ -6404,19 +6408,19 @@
         <v>76</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH46" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI46" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ46" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK46" t="s" s="2">
         <v>76</v>
@@ -6433,10 +6437,10 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -6447,7 +6451,7 @@
         <v>77</v>
       </c>
       <c r="G47" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H47" t="s" s="2">
         <v>76</v>
@@ -6456,19 +6460,19 @@
         <v>76</v>
       </c>
       <c r="J47" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="N47" t="s" s="2">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
@@ -6518,19 +6522,19 @@
         <v>76</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH47" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI47" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ47" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK47" t="s" s="2">
         <v>76</v>
@@ -6547,10 +6551,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -6561,7 +6565,7 @@
         <v>77</v>
       </c>
       <c r="G48" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H48" t="s" s="2">
         <v>76</v>
@@ -6570,19 +6574,19 @@
         <v>76</v>
       </c>
       <c r="J48" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="N48" t="s" s="2">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="O48" s="2"/>
       <c r="P48" t="s" s="2">
@@ -6632,13 +6636,13 @@
         <v>76</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH48" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI48" t="s" s="2">
         <v>76</v>
@@ -6661,10 +6665,10 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -6675,7 +6679,7 @@
         <v>77</v>
       </c>
       <c r="G49" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H49" t="s" s="2">
         <v>76</v>
@@ -6684,22 +6688,22 @@
         <v>76</v>
       </c>
       <c r="J49" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="N49" t="s" s="2">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="O49" t="s" s="2">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="P49" t="s" s="2">
         <v>76</v>
@@ -6748,19 +6752,19 @@
         <v>76</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH49" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AI49" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ49" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK49" t="s" s="2">
         <v>76</v>
@@ -6777,12 +6781,12 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AN49">
-    <filterColumn colId="6">
+    <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
       </customFilters>
     </filterColumn>
-    <filterColumn colId="26">
+    <filterColumn colId="27">
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>

</xml_diff>